<commit_message>
SW FMEA: host supervision tests are not collected by CI (SWF-ACT-055)
test_supervision.py and test_input_freshness.py define plain pytest-style
classes; tools/test_runner.py (unittest loader) collects 0 tests from
them, so the unit_tests job does not run them. They pass when run by hand
(13 and 6 tests). Detection text on SWF-032.C3, SWF-034.C1, SWF-040.C1 and
SWF-043.C1 corrected (D8 kept: targeted test method, not proven); action
SWF-ACT-055 to make them collectable and prove them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z9RYsWKq48KyCn88R4xJt
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$86</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -943,7 +943,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>46 (42)</t>
+          <t>47 (43)</t>
         </is>
       </c>
     </row>
@@ -12509,7 +12509,7 @@
       <c r="R49" s="39" t="inlineStr"/>
       <c r="S49" s="39" t="inlineStr"/>
     </row>
-    <row r="50" ht="141" customHeight="1">
+    <row r="50" ht="168" customHeight="1">
       <c r="A50" s="40" t="n"/>
       <c r="B50" s="40" t="n"/>
       <c r="C50" s="40" t="n"/>
@@ -12565,7 +12565,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_supervision.py: TxBlockedMonitor baseline, rise while engaged and panda-reset tests, in CI unit tests on every PR. Targeted, not proven by mutation; the txRateExceeded and heartbeatLost branches in selfdrived.py have no test</t>
+            <t>• test_supervision.py: TxBlockedMonitor baseline, rise while engaged and panda-reset tests. NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted, not proven by mutation; the txRateExceeded and heartbeatLost branches in selfdrived.py have no test</t>
           </r>
           <r>
             <rPr>
@@ -13104,7 +13104,7 @@
       <c r="R53" s="48" t="inlineStr"/>
       <c r="S53" s="48" t="inlineStr"/>
     </row>
-    <row r="54" ht="276" customHeight="1">
+    <row r="54" ht="409" customHeight="1">
       <c r="A54" s="30" t="inlineStr">
         <is>
           <r>
@@ -13356,7 +13356,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_supervision.py (consecutive samples, single-sample absorption, 0.5 s bound with stale samples, engagement grace), in CI unit tests on every PR. Targeted at the cause, not proven by mutation</t>
+            <t>• test_supervision.py (13 tests: consecutive samples, single-sample absorption, 0.5 s bound with stale samples, engagement grace). NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted at the cause, not proven by mutation</t>
           </r>
           <r>
             <rPr>
@@ -13424,12 +13424,40 @@
             </rPr>
             <t>Panda status supervision per TSR-615, TSR-621 and TSR-626a: controlsMismatch within 2 samples and 0.5 s (time-based); safety model/parameter mismatch as NO_ENTRY from start instead of a 10 s grace; pandaStates older than 0.2 s treated as mismatch; immediate disable on heartbeatLost, rising safetyTxBlocked, txRateExceeded and any panda fault flag</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SWF-ACT-055 · detection
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Make the host supervision tests run in CI: test_supervision.py and test_input_freshness.py define plain classes, which tools/test_runner.py (unittest loader) collects as 0 tests. Derive them from unittest.TestCase (or the repo's test base class), check that the unit_tests job reports them, and prove them by a mutation of supervision.py and input_freshness.py so D can drop below 8</t>
+          </r>
         </is>
       </c>
       <c r="O54" s="38" t="inlineStr">
         <is>
           <t>open
-in progress</t>
+in progress
+open</t>
         </is>
       </c>
       <c r="P54" s="33" t="inlineStr">
@@ -15470,7 +15498,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_input_freshness.py (6 tests: bound per service, wall clock for selfdriveState, inputs not yet seen), in CI unit tests on every PR. Targeted at the gate logic, not proven by mutation; no test stops selfdrived while engaged</t>
+            <t>• test_input_freshness.py (6 tests: bound per service, wall clock for selfdriveState, inputs not yet seen). NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted at the gate logic, not proven by mutation; no test stops selfdrived while engaged</t>
           </r>
           <r>
             <rPr>
@@ -16640,7 +16668,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_input_freshness.py (bound per service on the log clock), in CI unit tests on every PR; targeted at the gate, not proven by mutation. No test stops modeld or plannerd while engaged</t>
+            <t>• test_input_freshness.py (bound per service on the log clock). NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted at the gate, not proven by mutation. No test stops modeld or plannerd while engaged</t>
           </r>
           <r>
             <rPr>
@@ -20733,7 +20761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22533,52 +22561,87 @@
       <c r="H46" s="60" t="inlineStr"/>
       <c r="I46" s="60" t="inlineStr"/>
     </row>
-    <row r="47" ht="73.5" customHeight="1">
+    <row r="47" ht="87" customHeight="1">
       <c r="A47" s="60" t="inlineStr">
         <is>
+          <t>SWF-ACT-055</t>
+        </is>
+      </c>
+      <c r="B47" s="60" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="C47" s="60" t="inlineStr">
+        <is>
+          <t>Make the host supervision tests run in CI: test_supervision.py and test_input_freshness.py define plain classes, which tools/test_runner.py (unittest loader) collects as 0 tests. Derive them from unittest.TestCase (or the repo's test base class), check that the unit_tests job reports them, and prove them by a mutation of supervision.py and input_freshness.py so D can drop below 8</t>
+        </is>
+      </c>
+      <c r="D47" s="60" t="inlineStr">
+        <is>
+          <t>Jherrod Thomas</t>
+        </is>
+      </c>
+      <c r="E47" s="60" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="F47" s="60" t="inlineStr">
+        <is>
+          <t>SWF-034.C1</t>
+        </is>
+      </c>
+      <c r="G47" s="60" t="inlineStr"/>
+      <c r="H47" s="60" t="inlineStr"/>
+      <c r="I47" s="60" t="inlineStr"/>
+    </row>
+    <row r="48" ht="73.5" customHeight="1">
+      <c r="A48" s="60" t="inlineStr">
+        <is>
           <t>SWF-ACT-054</t>
         </is>
       </c>
-      <c r="B47" s="60" t="inlineStr">
+      <c r="B48" s="60" t="inlineStr">
         <is>
           <t>design change</t>
         </is>
       </c>
-      <c r="C47" s="60" t="inlineStr">
+      <c r="C48" s="60" t="inlineStr">
         <is>
           <t>Pin an opendbc commit that contains jherrodthomas/opendbc#15 (ATC-20, SWSR-518 amended per DQ-079; ATC-26, SWSR-311 amended per DQ-080), with its impact records moved to Integrated, and re-rate SWF-054 and SWF-055 at the new baseline. The fork merged it as 9859cb0 (master 515b9a2 also carries opendbc#16); the LionDriver pin is still 9a13f60</t>
         </is>
       </c>
-      <c r="D47" s="60" t="inlineStr">
+      <c r="D48" s="60" t="inlineStr">
         <is>
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E47" s="60" t="inlineStr">
+      <c r="E48" s="60" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="F47" s="60" t="inlineStr">
+      <c r="F48" s="60" t="inlineStr">
         <is>
           <t>SWF-054.C1
 SWF-055.C1</t>
         </is>
       </c>
-      <c r="G47" s="60" t="inlineStr">
+      <c r="G48" s="60" t="inlineStr">
         <is>
           <t>10/3/4</t>
         </is>
       </c>
-      <c r="H47" s="63" t="inlineStr">
+      <c r="H48" s="63" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="I47" s="60" t="inlineStr"/>
+      <c r="I48" s="60" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I47"/>
+  <autoFilter ref="A1:I48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
SW FMEA: SWF-062.C1 occurrence 6 -> 8, as the other by-design gaps
The terminal driver-monitoring reaction is a by-design gap with no documented requirement
(FSR-040's safe state is not defined for this path) and no field-exposure evidence, which
is O 8 under RT-2 §2. SWF-083.C1 and the System FMEA's SFM-025.C1 rate the same kind of gap
at O 8. AP stays H (S10 O8 D9). Raised by the System FMEA session. AI-drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z9RYsWKq48KyCn88R4xJt
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -23056,7 +23056,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Upstream design; FSR-040 names a safe state that the FSC does not define for this path</t>
+            <t>• Upstream design; FSR-040 names a safe state that the FSC does not define for this path. Requirements not documented and no field-exposure evidence cited, so O 8 (RT-2 §2), as SWF-083.C1 and SFM-025.C1</t>
           </r>
           <r>
             <rPr>
@@ -23070,7 +23070,7 @@
         </is>
       </c>
       <c r="J99" s="45" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K99" s="44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SW FMEA rev 1.1: HZ-013 end effects on SWF-035 and SWF-082 (F-37)
- SWF-035: the alert selection (priority, then start frame) masks the driver-monitoring
  escalation as it masks the takeover alert: driverDistracted2 / driverUnresponsive2 (MID)
  under speedTooHigh, the level 3 alerts (HIGH) under aeb or fcw (HIGHEST) or a later-starting
  HIGH alert. C1 extended with the DM priorities (events.py:532-563).
- SWF-082: soundd and ui carry the driver-monitoring alerts, so a process not running and not
  reported also leaves those alerts unpresented. The forced stop does not depend on either.
- Ratings unchanged. Removes the two SG-08 lint warnings on these modes; fta-fmea-mapping.md
  F-37 now leaves only the System FMEA's SFM-026 and SFM-027 without HZ-013.
AI-drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z9RYsWKq48KyCn88R4xJt
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -13685,7 +13685,7 @@
       <c r="R56" s="48" t="inlineStr"/>
       <c r="S56" s="48" t="inlineStr"/>
     </row>
-    <row r="57" ht="141" customHeight="1">
+    <row r="57" ht="208.5" customHeight="1">
       <c r="A57" s="49" t="inlineStr">
         <is>
           <r>
@@ -13791,6 +13791,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-013 (a driver-monitoring escalation masked, so an inattentive driver is not told; the forced stop still follows)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -13832,7 +13858,8 @@
       <c r="D57" s="50" t="inlineStr">
         <is>
           <t>HZ-012
-HZ-004</t>
+HZ-004
+HZ-013</t>
         </is>
       </c>
       <c r="E57" s="51" t="n">
@@ -13874,7 +13901,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Selection is by priority, then start frame (alertmanager.py:63). SoftDisableAlert is Priority.MID (events.py:161-166), below speedTooHigh (WARNING, HIGH, promptRepeat, events.py:995-1000), aeb/stockAeb (PERMANENT, HIGHEST, no sound, events.py:471-485) and driverDistracted3/driverUnresponsive3 (HIGH); the takeover text and warningSoft can be hidden for the first 2.5 s and only the last 0.5 s becomes ImmediateDisableAlert (events.py:224-228)</t>
+            <t>Selection is by priority, then start frame (alertmanager.py:63). SoftDisableAlert is Priority.MID (events.py:161-166), below speedTooHigh (WARNING, HIGH, promptRepeat, events.py:995-1000), aeb/stockAeb (PERMANENT, HIGHEST, no sound, events.py:471-485) and driverDistracted3/driverUnresponsive3 (HIGH); the takeover text and warningSoft can be hidden for the first 2.5 s and only the last 0.5 s becomes ImmediateDisableAlert (events.py:224-228). The same rule masks the driver-monitoring escalation: driverDistracted2 / driverUnresponsive2 (MID, events.py:532-563) under speedTooHigh, and the level 3 alerts (HIGH) under aeb or fcw (HIGHEST) or a later-starting HIGH alert</t>
           </r>
         </is>
       </c>
@@ -29076,7 +29103,7 @@
       <c r="R130" s="48" t="inlineStr"/>
       <c r="S130" s="48" t="inlineStr"/>
     </row>
-    <row r="131" ht="127.5" customHeight="1">
+    <row r="131" ht="181.5" customHeight="1">
       <c r="A131" s="49" t="inlineStr">
         <is>
           <r>
@@ -29156,6 +29183,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-013 (driver-monitoring alerts not presented when soundd or ui is not running; the forced stop does not depend on them)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -29196,7 +29249,8 @@
       </c>
       <c r="D131" s="50" t="inlineStr">
         <is>
-          <t>HZ-012</t>
+          <t>HZ-012
+HZ-013</t>
         </is>
       </c>
       <c r="E131" s="51" t="n">

</xml_diff>

<commit_message>
SW FMEA rev 1.3: lead answers DQ-342, DQ-366, DQ-365 applied; SWF-088 EPS-fault warning; SWF-ACT-055 in progress
- SWF-088 (new SWF-FN-055 on SWF-SE-054, car_events.py): EPS-fault warning latched at the low-priority prompt (C1, TSR-607 (b))
  or absent while the driver keeps steering (C2, TSR-607 (c)); O8 D10 AP H at BL-005; backs FTA BE-2.08 with SFM-038.
  SWF-ACT-077 completed after BL-005 (#174, #179), revised O3 D8 AP H as a prediction.
- SWF-062.C1 and SWF-ACT-059: SG-010 safe state decided (DQ-365 A, TSR-633), not implemented; action open.
- SWF-ACT-055 in progress: host supervision tests run in CI since #179 (1555 passed); D stays 8 until mutation.
- WP-W-04 v1.0, fmea-plan §3.3, fta-fmea-mapping F-28; generated outputs regenerated with the tools.

AI-drafted, not reviewed independently.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z9RYsWKq48KyCn88R4xJt
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Worksheet'!$A$2:$S$140</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Worksheet'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Actions'!$A$1:$I$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structure'!$A$1:$E$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1.2 · draft</t>
+          <t>1.3 · draft</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17">
@@ -946,7 +946,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>68 (64)</t>
+          <t>69 (64)</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S138"/>
+  <dimension ref="A1:S140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12512,7 +12512,7 @@
       <c r="R49" s="39" t="inlineStr"/>
       <c r="S49" s="39" t="inlineStr"/>
     </row>
-    <row r="50" ht="168" customHeight="1">
+    <row r="50" ht="154.5" customHeight="1">
       <c r="A50" s="40" t="n"/>
       <c r="B50" s="40" t="n"/>
       <c r="C50" s="40" t="n"/>
@@ -12568,7 +12568,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_supervision.py: TxBlockedMonitor baseline, rise while engaged and panda-reset tests. NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted, not proven by mutation; the txRateExceeded and heartbeatLost branches in selfdrived.py have no test</t>
+            <t>• test_supervision.py: TxBlockedMonitor baseline, rise while engaged and panda-reset tests. Not run in CI at BL-005 (plain classes, collected as 0 tests; passed by hand 2026-10-16); run in CI since #179 (487d4ef, SWF-ACT-055). Targeted, not proven by mutation; the txRateExceeded and heartbeatLost branches in selfdrived.py have no test</t>
           </r>
           <r>
             <rPr>
@@ -13359,7 +13359,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_supervision.py (13 tests: consecutive samples, single-sample absorption, 0.5 s bound with stale samples, engagement grace). NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted at the cause, not proven by mutation</t>
+            <t>• test_supervision.py (13 tests: consecutive samples, single-sample absorption, 0.5 s bound with stale samples, engagement grace). Not run in CI at BL-005 (plain classes, collected as 0 tests; passed by hand 2026-10-16); run in CI since #179 (487d4ef, SWF-ACT-055). Targeted at the cause, not proven by mutation</t>
           </r>
           <r>
             <rPr>
@@ -13460,7 +13460,7 @@
         <is>
           <t>open
 in progress
-open</t>
+in progress</t>
         </is>
       </c>
       <c r="P54" s="33" t="inlineStr">
@@ -15528,7 +15528,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_input_freshness.py (6 tests: bound per service, wall clock for selfdriveState, inputs not yet seen). NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted at the gate logic, not proven by mutation; no test stops selfdrived while engaged</t>
+            <t>• test_input_freshness.py (6 tests: bound per service, wall clock for selfdriveState, inputs not yet seen). Not run in CI at BL-005 (plain classes, collected as 0 tests; passed by hand 2026-10-16); run in CI since #179 (487d4ef, SWF-ACT-055). Targeted at the gate logic, not proven by mutation; no test stops selfdrived while engaged</t>
           </r>
           <r>
             <rPr>
@@ -16698,7 +16698,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• test_input_freshness.py (bound per service on the log clock). NOT run in CI: plain pytest-style classes, which tools/test_runner.py (unittest) collects as 0 tests; pass when run by hand at BL-005 (2026-10-16) (SWF-ACT-055). Targeted at the gate, not proven by mutation. No test stops modeld or plannerd while engaged</t>
+            <t>• test_input_freshness.py (bound per service on the log clock). Not run in CI at BL-005 (plain classes, collected as 0 tests; passed by hand 2026-10-16); run in CI since #179 (487d4ef, SWF-ACT-055). Targeted at the gate, not proven by mutation. No test stops modeld or plannerd while engaged</t>
           </r>
           <r>
             <rPr>
@@ -22909,7 +22909,7 @@
       <c r="R98" s="48" t="inlineStr"/>
       <c r="S98" s="48" t="inlineStr"/>
     </row>
-    <row r="99" ht="114" customHeight="1">
+    <row r="99" ht="154.5" customHeight="1">
       <c r="A99" s="49" t="inlineStr">
         <is>
           <r>
@@ -23071,7 +23071,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>By design the six driver-monitoring events are PERMANENT alerts only, with no SOFT_DISABLE or IMMEDIATE_DISABLE (events.py:524-570); the terminal reaction is the forced deceleration with lateral control kept. Whether that is the SG-010 safe state of FSR-040 is not recorded; it is queued for the lead (DQ-365, which absorbed DQ-220)</t>
+            <t>By design the six driver-monitoring events are PERMANENT alerts only, with no SOFT_DISABLE or IMMEDIATE_DISABLE (events.py:524-570); the terminal reaction is the forced deceleration with lateral control kept. The SG-010 safe state is decided (DQ-365 A, which absorbed DQ-220; TSR-633) as stop in lane, stay stopped and held, re-engagement locked out until the driver responds. The code does not hold at standstill or lock out until a later disengagement (TSR-633 not met)</t>
           </r>
         </is>
       </c>
@@ -23083,7 +23083,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• Upstream design; FSR-040 names a safe state that the FSC does not define for this path. Requirements not documented and no field-exposure evidence cited, so O 8 (RT-2 §2), as SWF-083.C1 and SFM-025.C1</t>
+            <t>• Upstream design; the safe state is now defined (TSR-633, DQ-365 A) but not implemented. No field-exposure evidence cited, so O 8 (RT-2 §2), as SWF-083.C1 and SFM-025.C1</t>
           </r>
           <r>
             <rPr>
@@ -23146,13 +23146,13 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Define the SG-010 safe state for FSR-040 (lead decision DQ-365, which absorbed DQ-220) and, if it differs from the current forced deceleration with lateral kept, implement it with a terminal-alert test</t>
-          </r>
-        </is>
-      </c>
-      <c r="O99" s="59" t="inlineStr">
-        <is>
-          <t>decision pending</t>
+            <t>Implement the SG-010 safe state decided in DQ-365 (A, which absorbed DQ-220; TSR-633): after the forced deceleration keep the vehicle stopped and held and lock out re-engagement and resumption until the driver responds; add a terminal-alert test that checks standstill, hold and lockout</t>
+          </r>
+        </is>
+      </c>
+      <c r="O99" s="53" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
       <c r="P99" s="43" t="inlineStr"/>
@@ -30547,7 +30547,7 @@
       <c r="R136" s="39" t="inlineStr"/>
       <c r="S136" s="39" t="inlineStr"/>
     </row>
-    <row r="137" ht="235.5" customHeight="1">
+    <row r="137" ht="262.5" customHeight="1">
       <c r="A137" s="42" t="n"/>
       <c r="B137" s="42" t="n"/>
       <c r="C137" s="42" t="n"/>
@@ -30642,7 +30642,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Define the SG-010 safe state for FSR-040 (lead decision DQ-365, which absorbed DQ-220) and, if it differs from the current forced deceleration with lateral kept, implement it with a terminal-alert test</t>
+            <t>Implement the SG-010 safe state decided in DQ-365 (A, which absorbed DQ-220; TSR-633): after the forced deceleration keep the vehicle stopped and held and lock out re-engagement and resumption until the driver responds; add a terminal-alert test that checks standstill, hold and lockout</t>
           </r>
           <r>
             <rPr>
@@ -30673,9 +30673,9 @@
           </r>
         </is>
       </c>
-      <c r="O137" s="59" t="inlineStr">
-        <is>
-          <t>decision pending
+      <c r="O137" s="53" t="inlineStr">
+        <is>
+          <t>open
 open</t>
         </is>
       </c>
@@ -30926,9 +30926,367 @@
       <c r="R138" s="48" t="inlineStr"/>
       <c r="S138" s="48" t="inlineStr"/>
     </row>
+    <row r="139" ht="127.5" customHeight="1">
+      <c r="A139" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SWF-SE-054
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>card main loop and stock AEB interlock</t>
+          </r>
+        </is>
+      </c>
+      <c r="B139" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SWF-FN-055
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Raise the EPS-fault warning while engaged (TSR-607); the take-over request, with the lighter prompt only for the first 1.5 s after an override or at standstill, and at least the lighter prompt when the fault lasts over 1.5 s while the driver keeps steering</t>
+          </r>
+        </is>
+      </c>
+      <c r="C139" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Driver not prompted to take over while lateral control is lost; lane departure (counterpart of SFM-038.C1)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Next higher  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The item stays engaged with lateral assist lost; the envelope refuses lateral frames (EPS-fault refusal, reference build) and the panda siren sounds after about 1 s of a persistent fault while authority is granted</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">Local  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>steerTempUnavailableSilent (LOW priority, small alert with prompt chime, no soft disable; events.py:516-521) instead of steerTempUnavailable (soft disable), or no EPS event at all while the driver keeps steering</t>
+          </r>
+        </is>
+      </c>
+      <c r="D139" s="31" t="inlineStr">
+        <is>
+          <t>HZ-004</t>
+        </is>
+      </c>
+      <c r="E139" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F139" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SWF-088 · late
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>EPS-fault warning held at the low-priority prompt, or not given, for the whole of a temporary EPS fault while engaged</t>
+          </r>
+        </is>
+      </c>
+      <c r="G139" s="33" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="H139" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>By design at BL-005, after a steering override in the last 1.5 s or at standstill, a temporary EPS fault raises only steerTempUnavailableSilent and silent_steer_warning stays latched while the fault lasts, so a long fault never escalates to the take-over request (car_events.py:162-177; TSR-607 (b), DQ-342 A; GAP-03)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I139" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream openpilot design (a softer alert after an override); TSR-607 (b) not implemented at BL-005, so O 8 (RT-2 §2), as the other by-design gaps</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/car/car_events.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="J139" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K139" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No test of the EPS-fault events at BL-005</t>
+          </r>
+        </is>
+      </c>
+      <c r="L139" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="M139" s="37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N139" s="34" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SWF-ACT-077 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Escalate the EPS-fault warning per TSR-607 (DQ-342 A, DQ-366 A): allow steerTempUnavailableSilent only for the first 1.5 s of the fault (steer_fault_frames, STEER_FAULT_SILENT_FRAMES), then the take-over request; give at least the lighter prompt when the fault lasts over 1.5 s while the driver keeps steering; unit tests</t>
+          </r>
+        </is>
+      </c>
+      <c r="O139" s="56" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="P139" s="33" t="inlineStr">
+        <is>
+          <t>10/3/8</t>
+        </is>
+      </c>
+      <c r="Q139" s="37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="R139" s="39" t="inlineStr"/>
+      <c r="S139" s="39" t="inlineStr"/>
+    </row>
+    <row r="140" ht="127.5" customHeight="1">
+      <c r="A140" s="42" t="n"/>
+      <c r="B140" s="42" t="n"/>
+      <c r="C140" s="42" t="n"/>
+      <c r="D140" s="42" t="n"/>
+      <c r="E140" s="42" t="n"/>
+      <c r="F140" s="42" t="n"/>
+      <c r="G140" s="43" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="H140" s="44" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>By design at BL-005, a temporary EPS fault that starts while the driver is steering raises no EPS event while they keep steering (no_steer_warning, car_events.py:164-166); the take-over request follows only on release (TSR-607 (c), DQ-366 A)</t>
+          </r>
+        </is>
+      </c>
+      <c r="I140" s="44" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• Upstream openpilot design; TSR-607 (c) not implemented at BL-005, so O 8 (RT-2 §2)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="005B6676"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+   openpilot/selfdrive/car/car_events.py</t>
+          </r>
+        </is>
+      </c>
+      <c r="J140" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="K140" s="44" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="008A5A00"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• No test of the EPS-fault events at BL-005</t>
+          </r>
+        </is>
+      </c>
+      <c r="L140" s="54" t="n">
+        <v>10</v>
+      </c>
+      <c r="M140" s="52" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N140" s="44" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="001F4E8C"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">SWF-ACT-077 · design change
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Escalate the EPS-fault warning per TSR-607 (DQ-342 A, DQ-366 A): allow steerTempUnavailableSilent only for the first 1.5 s of the fault (steer_fault_frames, STEER_FAULT_SILENT_FRAMES), then the take-over request; give at least the lighter prompt when the fault lasts over 1.5 s while the driver keeps steering; unit tests</t>
+          </r>
+        </is>
+      </c>
+      <c r="O140" s="47" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="P140" s="43" t="inlineStr">
+        <is>
+          <t>10/3/8</t>
+        </is>
+      </c>
+      <c r="Q140" s="52" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="R140" s="48" t="inlineStr"/>
+      <c r="S140" s="48" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:S138"/>
-  <mergeCells count="226">
+  <autoFilter ref="A2:S140"/>
+  <mergeCells count="232">
     <mergeCell ref="C30:C31"/>
     <mergeCell ref="E92:E93"/>
     <mergeCell ref="B124:B126"/>
@@ -30993,6 +31351,7 @@
     <mergeCell ref="B58:B59"/>
     <mergeCell ref="A90:A91"/>
     <mergeCell ref="F49:F51"/>
+    <mergeCell ref="D139:D140"/>
     <mergeCell ref="E128:E129"/>
     <mergeCell ref="C100:C101"/>
     <mergeCell ref="F116:F118"/>
@@ -31002,7 +31361,9 @@
     <mergeCell ref="A96:A98"/>
     <mergeCell ref="C96:C98"/>
     <mergeCell ref="F22:F23"/>
+    <mergeCell ref="A139:A140"/>
     <mergeCell ref="B60:B61"/>
+    <mergeCell ref="C139:C140"/>
     <mergeCell ref="B69:B70"/>
     <mergeCell ref="B76:B78"/>
     <mergeCell ref="B3:B5"/>
@@ -31049,6 +31410,7 @@
     <mergeCell ref="F96:F98"/>
     <mergeCell ref="E20:E21"/>
     <mergeCell ref="E60:E61"/>
+    <mergeCell ref="F139:F140"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="E69:E70"/>
     <mergeCell ref="E76:E78"/>
@@ -31087,6 +31449,7 @@
     <mergeCell ref="E134:E135"/>
     <mergeCell ref="D20:D21"/>
     <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E139:E140"/>
     <mergeCell ref="F14:F15"/>
     <mergeCell ref="B116:B118"/>
     <mergeCell ref="E87:E89"/>
@@ -31131,6 +31494,7 @@
     <mergeCell ref="E45:E46"/>
     <mergeCell ref="D96:D98"/>
     <mergeCell ref="A103:A105"/>
+    <mergeCell ref="B139:B140"/>
     <mergeCell ref="C103:C105"/>
     <mergeCell ref="D58:D59"/>
     <mergeCell ref="F58:F59"/>
@@ -31157,7 +31521,7 @@
     <mergeCell ref="D22:D23"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87 R88 R89 R90 R91 R92 R93 R94 R95 R96 R97 R98 R99 R100 R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R116 R117 R118 R119 R120 R121 R122 R123 R124 R125 R126 R127 R128 R129 R130 R131 R132 R133 R134 R135 R136 R137 R138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
+    <dataValidation sqref="R3 R4 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87 R88 R89 R90 R91 R92 R93 R94 R95 R96 R97 R98 R99 R100 R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R116 R117 R118 R119 R120 R121 R122 R123 R124 R125 R126 R127 R128 R129 R130 R131 R132 R133 R134 R135 R136 R137 R138 R139 R140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Review" prompt="Reviewer decision for this cause" type="list">
       <formula1>"Agree,Re-rate,Reject,Question"</formula1>
     </dataValidation>
   </dataValidations>
@@ -31165,7 +31529,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSW FMEA — safety-relevant software elements · rev 1.2 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSW FMEA — safety-relevant software elements · rev 1.3 · BL-005&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -31180,7 +31544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33013,7 +33377,7 @@
       </c>
       <c r="E47" s="61" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>in progress</t>
         </is>
       </c>
       <c r="F47" s="61" t="inlineStr">
@@ -33023,7 +33387,11 @@
       </c>
       <c r="G47" s="61" t="inlineStr"/>
       <c r="H47" s="61" t="inlineStr"/>
-      <c r="I47" s="61" t="inlineStr"/>
+      <c r="I47" s="61" t="inlineStr">
+        <is>
+          <t>Run in CI: #179 (487d4ef, 2026-10-17) derives both from unittest.TestCase; the unit_tests job of tests run 38991473673 reports 1555 passed (1535 before: 19 newly collected and 1 new EPS test). Mutation proof not done, so D stays 8</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="73.5" customHeight="1">
       <c r="A48" s="61" t="inlineStr">
@@ -33183,7 +33551,7 @@
       <c r="H51" s="61" t="inlineStr"/>
       <c r="I51" s="61" t="inlineStr"/>
     </row>
-    <row r="52" ht="46.5" customHeight="1">
+    <row r="52" ht="73.5" customHeight="1">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>SWF-ACT-059</t>
@@ -33196,7 +33564,7 @@
       </c>
       <c r="C52" s="61" t="inlineStr">
         <is>
-          <t>Define the SG-010 safe state for FSR-040 (lead decision DQ-365, which absorbed DQ-220) and, if it differs from the current forced deceleration with lateral kept, implement it with a terminal-alert test</t>
+          <t>Implement the SG-010 safe state decided in DQ-365 (A, which absorbed DQ-220; TSR-633): after the forced deceleration keep the vehicle stopped and held and lock out re-engagement and resumption until the driver responds; add a terminal-alert test that checks standstill, hold and lockout</t>
         </is>
       </c>
       <c r="D52" s="61" t="inlineStr">
@@ -33206,7 +33574,7 @@
       </c>
       <c r="E52" s="61" t="inlineStr">
         <is>
-          <t>decision pending</t>
+          <t>open</t>
         </is>
       </c>
       <c r="F52" s="61" t="inlineStr">
@@ -33838,8 +34206,56 @@
       <c r="H69" s="61" t="inlineStr"/>
       <c r="I69" s="61" t="inlineStr"/>
     </row>
+    <row r="70" ht="100.5" customHeight="1">
+      <c r="A70" s="61" t="inlineStr">
+        <is>
+          <t>SWF-ACT-077</t>
+        </is>
+      </c>
+      <c r="B70" s="61" t="inlineStr">
+        <is>
+          <t>design change</t>
+        </is>
+      </c>
+      <c r="C70" s="61" t="inlineStr">
+        <is>
+          <t>Escalate the EPS-fault warning per TSR-607 (DQ-342 A, DQ-366 A): allow steerTempUnavailableSilent only for the first 1.5 s of the fault (steer_fault_frames, STEER_FAULT_SILENT_FRAMES), then the take-over request; give at least the lighter prompt when the fault lasts over 1.5 s while the driver keeps steering; unit tests</t>
+        </is>
+      </c>
+      <c r="D70" s="61" t="inlineStr">
+        <is>
+          <t>Jherrod Thomas</t>
+        </is>
+      </c>
+      <c r="E70" s="62" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F70" s="61" t="inlineStr">
+        <is>
+          <t>SWF-088.C1
+SWF-088.C2</t>
+        </is>
+      </c>
+      <c r="G70" s="61" t="inlineStr">
+        <is>
+          <t>10/3/8</t>
+        </is>
+      </c>
+      <c r="H70" s="63" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="I70" s="61" t="inlineStr">
+        <is>
+          <t>#174 (7158a9a) and #179 (487d4ef): openpilot/selfdrive/car/car_events.py:17, 169-187; openpilot/selfdrive/car/tests/test_steer_fault_warning.py (7 tests, unittest, collected by the unit_tests job); impact record assurance/07-supporting/impact/change-2026-10-17-eps-fault-escalation.md. Implemented and unit-tested after BL-005, not verified on the vehicle and not proven by mutation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I69"/>
+  <autoFilter ref="A1:I70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -34909,7 +35325,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="33" customHeight="1">
+    <row r="41" ht="73.5" customHeight="1">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>SWF-SE-054</t>
@@ -34932,7 +35348,8 @@
       </c>
       <c r="E41" s="61" t="inlineStr">
         <is>
-          <t>SWF-FN-054: Run the car interface every CAN cycle, publish carState, and actuate only the latest carControl</t>
+          <t>SWF-FN-054: Run the car interface every CAN cycle, publish carState, and actuate only the latest carControl
+SWF-FN-055: Raise the EPS-fault warning while engaged (TSR-607); the take-over request, with the lighter prompt only for the first 1.5 s after an override or at standstill, and at least the lighter prompt when the fault lasts over 1.5 s while the driver keeps steering</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SW FMEA: HZ-006 effects on SWF-055 and SWF-089 (FTA BE-1.25, SG-04)
WP-A-04 v1.12 cites BE-1.25 in the SG-04 tree. An authority grant covers
longitudinal commands, so SWF-055 and SWF-089 gain HZ-006 end effects,
as SWF-007 has. SWF-002 is steering-only and stays HZ-001; its note says
why, and points at SWF-007..009 for the controls_allowed part. Ratings
unchanged. Review md, xlsx and fig 3-6 regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z9RYsWKq48KyCn88R4xJt
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -20335,7 +20335,7 @@
       <c r="R85" s="48" t="inlineStr"/>
       <c r="S85" s="48" t="inlineStr"/>
     </row>
-    <row r="86" ht="235.5" customHeight="1">
+    <row r="86" ht="289.5" customHeight="1">
       <c r="A86" s="49" t="inlineStr">
         <is>
           <r>
@@ -20441,6 +20441,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-006 (the regained authority passes longitudinal commands too; braking without the driver's engagement, HE-04.4)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -20482,7 +20508,8 @@
       <c r="D86" s="50" t="inlineStr">
         <is>
           <t>HZ-010
-HZ-002</t>
+HZ-002
+HZ-006</t>
         </is>
       </c>
       <c r="E86" s="51" t="n">
@@ -31362,7 +31389,7 @@
       <c r="R140" s="48" t="inlineStr"/>
       <c r="S140" s="48" t="inlineStr"/>
     </row>
-    <row r="141" ht="154.5" customHeight="1">
+    <row r="141" ht="208.5" customHeight="1">
       <c r="A141" s="49" t="inlineStr">
         <is>
           <r>
@@ -31442,6 +31469,32 @@
               <color rgb="005B6676"/>
               <sz val="9"/>
             </rPr>
+            <t xml:space="preserve">End  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Contributes to HZ-006 (the grant covers longitudinal commands; braking without the driver's engagement for up to the 150 ms tolerance, HE-04.4)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="005B6676"/>
+              <sz val="9"/>
+            </rPr>
             <t xml:space="preserve">Next higher  </t>
           </r>
           <r>
@@ -31482,7 +31535,8 @@
       </c>
       <c r="D141" s="50" t="inlineStr">
         <is>
-          <t>HZ-010</t>
+          <t>HZ-010
+HZ-006</t>
         </is>
       </c>
       <c r="E141" s="51" t="n">

</xml_diff>

<commit_message>
DQ-300: no drive requested while the car reports a stock AEB event
While carState.stockAeb is true, controlsd caps the longitudinal target and
the upper PID limit at 0 m/s^2 (stock_aeb_stand_down in longcontrol.py), so
actuators.accel is at most 0 from the first frame of the event; a braking
request still passes. DQ-300 A (lead, 2026-10-18), System FMEA SFM-ACT-020.
The AOU-04R vehicle test still runs.

- 4 tests in selfdrive/controls/tests/test_stock_aeb.py, including the
  reference car's controller wound up before the event
- change record change-2026-10-19-stock-aeb-stand-down and index row; the
  opendbc Toyota controller's rate limit and positive terms are noted (OI-2)
- controlsd.py:N and longcontrol.py:N references in the living documents
  moved with the code; generated files regenerated

AI-drafted (I0); not reviewed independently.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y4mHLRpHEhwhLgfhGm6KK8
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -15207,7 +15207,7 @@
               <sz val="8"/>
             </rPr>
             <t xml:space="preserve">
-   openpilot/selfdrive/controls/controlsd.py:194</t>
+   openpilot/selfdrive/controls/controlsd.py:195</t>
           </r>
         </is>
       </c>
@@ -17303,7 +17303,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>At BL-004 self.desired_curvature and the torque PID integrator became NaN and stayed NaN, the sanitiser replaced the outputs with 0 and only logged. At BL-005 the step with a non-finite input runs with latActive or longActive false and the controllers reset (controlsd.py:122-131, 141-144, 154-159); the output is zero for as long as the input stays non-finite, without an event</t>
+            <t>At BL-004 self.desired_curvature and the torque PID integrator became NaN and stayed NaN, the sanitiser replaced the outputs with 0 and only logged. At BL-005 the step with a non-finite input runs with latActive or longActive false and the controllers reset (controlsd.py:122-131, 141-144, 155-160); the output is zero for as long as the input stays non-finite, without an event</t>
           </r>
         </is>
       </c>
@@ -17353,7 +17353,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>A NaN desired curvature (modelV2 or lateralManeuverPlan) or roll. At BL-004 it latched self.desired_curvature and the PID integrator for the drive (reproduced with the BL-004 clip_curvature and PIDController in isolation, scratch probe). Since #51 (BL-005) the step runs with latActive false, the controller is reset and desired_curvature is reset if non-finite (controlsd.py:122-128, 141-142, 154-155), so the latch is gone. Remaining: a persistent non-finite input silently zeroes lateral output while the item shows engaged, with no event or alert (TSR-604 asks an immediate disable; IA host-supervision OI-4); other inputs (vEgo, curvature from carState, vehicleParameters) are not guarded</t>
+            <t>A NaN desired curvature (modelV2 or lateralManeuverPlan) or roll. At BL-004 it latched self.desired_curvature and the PID integrator for the drive (reproduced with the BL-004 clip_curvature and PIDController in isolation, scratch probe). Since #51 (BL-005) the step runs with latActive false, the controller is reset and desired_curvature is reset if non-finite (controlsd.py:122-128, 141-142, 155-156), so the latch is gone. Remaining: a persistent non-finite input silently zeroes lateral output while the item shows engaged, with no event or alert (TSR-604 asks an immediate disable; IA host-supervision OI-4); other inputs (vEgo, curvature from carState, vehicleParameters) are not guarded</t>
           </r>
         </is>
       </c>
@@ -17498,7 +17498,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>A NaN aTarget made the LongControl PID integrator NaN even with ki=0 (0·NaN), so accel stayed NaN, sanitised to 0, until the state machine left pid (longcontrol.py:56-71). Since #51 (BL-005) a non-finite aTarget sets longActive false and 0 is passed instead, and LongControl is reset (controlsd.py:129-131, 143-144). Remaining: zero acceleration request, no event, while the input stays non-finite</t>
+            <t>A NaN aTarget made the LongControl PID integrator NaN even with ki=0 (0·NaN), so accel stayed NaN, sanitised to 0, until the state machine left pid (longcontrol.py:65-80). Since #51 (BL-005) a non-finite aTarget sets longActive false and 0 is passed instead, and LongControl is reset (controlsd.py:129-131, 143-144). Remaining: zero acceleration request, no event, while the input stays non-finite</t>
           </r>
         </is>
       </c>
@@ -17812,7 +17812,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>The 4 m/s³ windup/winddown limit is applied before the pitch compensation and the PID (carcontroller.py:197-238), so the sent command has no rate limit; pitch comes from CC.orientationNED, which controlsd fills from deviceMotion with no validity check (controlsd.py:69-71, 157-159)</t>
+            <t>The 4 m/s³ windup/winddown limit is applied before the pitch compensation and the PID (carcontroller.py:197-238), so the sent command has no rate limit; pitch comes from CC.orientationNED, which controlsd fills from deviceMotion with no validity check (controlsd.py:69-71, 158-160)</t>
           </r>
         </is>
       </c>
@@ -18172,7 +18172,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>controlsd raises on input it does not guard and exits; the 100 Hz loop has no exception handling. The example of BL-004, int(NaN) when lateralDelay is not finite (latcontrol_torque.py:100), is guarded since #51 (falls back to steerActuatorDelay, controlsd.py:157-159); other inputs are not</t>
+            <t>controlsd raises on input it does not guard and exits; the 100 Hz loop has no exception handling. The example of BL-004, int(NaN) when lateralDelay is not finite (latcontrol_torque.py:100), is guarded since #51 (falls back to steerActuatorDelay, controlsd.py:158-160); other inputs are not</t>
           </r>
         </is>
       </c>
@@ -18299,7 +18299,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Loop overrun or scheduling delay (Python, CTRL_HIGH on core 4, controlsd.py:237); Ratekeeper only monitors (228-233) and the loop is paced by selfdriveState; card actuates the latest carControl each CAN cycle as long as it is alive within 10 periods (card.py:234; cereal/messaging/__init__.py:265)</t>
+            <t>Loop overrun or scheduling delay (Python, CTRL_HIGH on core 4, controlsd.py:238); Ratekeeper only monitors (228-233) and the loop is paced by selfdriveState; card actuates the latest carControl each CAN cycle as long as it is alive within 10 periods (card.py:234; cereal/messaging/__init__.py:265)</t>
           </r>
         </is>
       </c>
@@ -18714,7 +18714,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>cancel = CS.cruiseState.enabled and not CC.enabled (controlsd.py:162), where CC.enabled is the unchecked selfdriveState (SWF-040.C1), and it is sent only inside the 33 Hz ACC_CONTROL frame (carcontroller.py:187, 253) while card is actuating. The selfdrived backstop does nothing: cruiseMismatch fires after 6 s (selfdrived.py:425-428) but has no alert or disable type (events.py:458-460, commented out)</t>
+            <t>cancel = CS.cruiseState.enabled and not CC.enabled (controlsd.py:163), where CC.enabled is the unchecked selfdriveState (SWF-040.C1), and it is sent only inside the 33 Hz ACC_CONTROL frame (carcontroller.py:187, 253) while card is actuating. The selfdrived backstop does nothing: cruiseMismatch fires after 6 s (selfdrived.py:425-428) but has no alert or disable type (events.py:458-460, commented out)</t>
           </r>
         </is>
       </c>
@@ -19186,7 +19186,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>forceDecel set in the same cycle as softDisabling or noResponseForceDecel (controlsd.py:235-236); the planner sets the cruise target to 0 at once (longitudinal_planner.py:84-85)</t>
+            <t>forceDecel set in the same cycle as softDisabling or noResponseForceDecel (controlsd.py:236-237); the planner sets the cruise target to 0 at once (longitudinal_planner.py:84-85)</t>
           </r>
         </is>
       </c>
@@ -19718,7 +19718,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>The Toyota CarController takes pcm_accel_cmd from actuators.accel with no longActive gate (carcontroller.py:197-250); the inactive value relies on LongControl returning 0 in its off state (longcontrol.py:56-58), so a defect or stale carControl upstream passes through</t>
+            <t>The Toyota CarController takes pcm_accel_cmd from actuators.accel with no longActive gate (carcontroller.py:197-250); the inactive value relies on LongControl returning 0 in its off state (longcontrol.py:65-67), so a defect or stale carControl upstream passes through</t>
           </r>
         </is>
       </c>
@@ -22396,7 +22396,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Unhandled exception: the loop has no exception handling (card.py:277-284). A non-finite torque or acceleration raises in the CarController (int(round(nan)), carcontroller.py:105; math.floor in packer.py:24); controlsd sanitises its actuators (controlsd.py:171-180), so the path needs a value made non-finite inside card (CarState or pitch compensation)</t>
+            <t>Unhandled exception: the loop has no exception handling (card.py:277-284). A non-finite torque or acceleration raises in the CarController (int(round(nan)), carcontroller.py:105; math.floor in packer.py:24); controlsd sanitises its actuators (controlsd.py:172-181), so the path needs a value made non-finite inside card (CarState or pitch compensation)</t>
           </r>
         </is>
       </c>
@@ -30494,7 +30494,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>The request crosses three processes with no freshness check on the flag: controlsd reads driverMonitoringState.noResponseForceDecel without an alive or valid check (controlsd.py:49-51, 235), and plannerd reads controlsState.forceDecel the same way (longitudinal_planner.py:84); its own valid flag is not read by controlsd (SWF-065.C1). A stopped dmonitoringd leaves the last value in place until selfdrived soft-disables (SWF-064)</t>
+            <t>The request crosses three processes with no freshness check on the flag: controlsd reads driverMonitoringState.noResponseForceDecel without an alive or valid check (controlsd.py:49-51, 236), and plannerd reads controlsState.forceDecel the same way (longitudinal_planner.py:84); its own valid flag is not read by controlsd (SWF-065.C1). A stopped dmonitoringd leaves the last value in place until selfdrived soft-disables (SWF-064)</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
SW FMEA rev 1.6: SWF-067.C1 D9 -> D8, SWF-ACT-063 completed
The CI unit_tests job runs again (LFS mirror back) and is green with
test_assured_config.py (tests run 39296172878 at 6126485: 1578 passed,
0 failed). SWF-067.C1 moves to D8, still AP H (targeted, not proven by
mutation); SWF-ACT-063 completed with that run as evidence. Totals
unchanged. Generated files rebuilt with the tools.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z9RYsWKq48KyCn88R4xJt
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1.5 · draft</t>
+          <t>1.6 · draft</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>71 (65)</t>
+          <t>71 (64)</t>
         </is>
       </c>
     </row>
@@ -24571,7 +24571,7 @@
       <c r="R106" s="48" t="inlineStr"/>
       <c r="S106" s="48" t="inlineStr"/>
     </row>
-    <row r="107" ht="154.5" customHeight="1">
+    <row r="107" ht="141" customHeight="1">
       <c r="A107" s="30" t="inlineStr">
         <is>
           <r>
@@ -24766,10 +24766,10 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <color rgb="008A5A00"/>
-              <sz val="10"/>
-            </rPr>
-            <t>• test_assured_config.py: each setting refuses entry, entry only, other platforms unchanged, distance button ignored on the reference platform. Collected by the CI unit_tests job but not yet run there (the scons jobs fail in setup on the git-lfs 404); run locally for #287 only. D 8 once CI runs it, D 4 with mutation</t>
+              <color rgb="001B2430"/>
+              <sz val="10"/>
+            </rPr>
+            <t>• test_assured_config.py: each setting refuses entry, entry only, other platforms unchanged, distance button ignored on the reference platform. Run by the CI unit_tests job since the LFS mirror returned (tests run 39296172878 at 6126485: 1578 passed, 0 failed); not proven by mutation, so D 8, D 4 with mutation</t>
           </r>
           <r>
             <rPr>
@@ -24782,8 +24782,8 @@
           </r>
         </is>
       </c>
-      <c r="L107" s="36" t="n">
-        <v>9</v>
+      <c r="L107" s="35" t="n">
+        <v>8</v>
       </c>
       <c r="M107" s="37" t="inlineStr">
         <is>
@@ -24812,9 +24812,9 @@
           </r>
         </is>
       </c>
-      <c r="O107" s="57" t="inlineStr">
-        <is>
-          <t>in progress</t>
+      <c r="O107" s="56" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="P107" s="33" t="inlineStr">
@@ -32263,7 +32263,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSW FMEA — safety-relevant software elements · rev 1.5 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSW FMEA — safety-relevant software elements · rev 1.6 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -34436,7 +34436,7 @@
       <c r="H55" s="61" t="inlineStr"/>
       <c r="I55" s="61" t="inlineStr"/>
     </row>
-    <row r="56" ht="154.5" customHeight="1">
+    <row r="56" ht="141" customHeight="1">
       <c r="A56" s="61" t="inlineStr">
         <is>
           <t>SWF-ACT-063</t>
@@ -34457,9 +34457,9 @@
           <t>Jherrod Thomas</t>
         </is>
       </c>
-      <c r="E56" s="61" t="inlineStr">
-        <is>
-          <t>in progress</t>
+      <c r="E56" s="62" t="inlineStr">
+        <is>
+          <t>completed</t>
         </is>
       </c>
       <c r="F56" s="61" t="inlineStr">
@@ -34479,7 +34479,7 @@
       </c>
       <c r="I56" s="61" t="inlineStr">
         <is>
-          <t>DQ-221 A implemented in #287 (69cddaa): assured_config.py (settings_in_scope), selfdrived.py (add_reference_entry_events, distance_button_pressed), events.py (settingNotAssured); tests in test_assured_config.py; change record assurance/07-supporting/impact/change-2026-10-19-reference-entry-checks.md. The tests ran locally only (the 22 of 24 that do not need the compiled Params library pass, per the #287 merge note); the CI unit_tests job has not run them (scons setup fails on the git-lfs 404). Completes when CI runs them; not verified in the vehicle (change record OI-5)</t>
+          <t>DQ-221 A implemented in #287 (69cddaa): assured_config.py (settings_in_scope), selfdrived.py (add_reference_entry_events, distance_button_pressed), events.py (settingNotAssured); tests in test_assured_config.py, collected by the CI unit_tests job and green there in tests run 39296172878 (6126485, 2026-10-19: 1578 passed, 0 failed); change record assurance/07-supporting/impact/change-2026-10-19-reference-entry-checks.md. Unit-tested, not proven by mutation and not verified in the vehicle (change record OI-5). Achieved: O5 D8 (rev 1.6)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SW FMEA rev 1.8: engaged-mismatch 0.3 s and siren cases since panda f4803c5 (text only)
From the FSC/TSC routes walk (#395), as the coordinator asked while the SW
FMEA has no active owner session. Changes:
- SWF-014, -020, -030, -036, -039, -040 and -048 described the engaged
  mismatch only as "about 3 s". They now also give the reference-build
  behaviour since panda f4803c5: revocation 0.3 s after the first
  not-engaged heartbeat (TSR-307(a)), and a siren 0.5 s later while PCM
  cruise stays on (TSR-516(c)). The plant numbers are from
  engaged-mismatch.md (synthetic, no credit).
- The SWF-014 and SWF-039 mechanisms now cover TSR-516(b) (DQ-404) and (c).
Ratings are unchanged. SWF-014, -036, -039, -040 and -048 carry an open note
that the re-rating is pending against the next baseline. fmea-plan v0.30.
AI-drafted; not reviewed independently.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142mASafXfhM7QmcnMZCDqi
</commit_message>
<xml_diff>
--- a/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
+++ b/assurance/08-analyses/fmea/exports/review/sw-fmea-review.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1.7 · draft</t>
+          <t>1.8 · draft</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>• TX arrival supervision in the 100 Hz safety task, started at the grant (safety.h tx_arrival_checks, toyota.h:599-606); timeouts from TSR-408, not yet confirmed on reference drive logs (IA tx-arrival OI-1). The engaged-mismatch path (about 3 s) is unchanged</t>
+            <t>• TX arrival supervision in the 100 Hz safety task, started at the grant (safety.h tx_arrival_checks, toyota.h:599-606); timeouts from TSR-408, not yet confirmed on reference drive logs (IA tx-arrival OI-1). The engaged-mismatch path (about 3 s at BL-006) revokes 0.3 s after the first not-engaged heartbeat since panda f4803c5, reference build, after BL-006 (TSR-307(a))</t>
           </r>
           <r>
             <rPr>
@@ -15300,7 +15300,7 @@
       <c r="R63" s="48" t="inlineStr"/>
       <c r="S63" s="48" t="inlineStr"/>
     </row>
-    <row r="64" ht="262.5" customHeight="1">
+    <row r="64" ht="289.5" customHeight="1">
       <c r="A64" s="49" t="inlineStr">
         <is>
           <r>
@@ -15414,7 +15414,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>Steering and acceleration continue with no supervision of model, localizer or comm faults; pandad drops heartbeat engaged after 0.1 s (pandad.cc:424) but the panda withdraws only after the engaged-mismatch count, about 3 s (panda main.c:226-232, SWF-014.C2)</t>
+            <t>Steering and acceleration continue with no supervision of model, localizer or comm faults; pandad drops heartbeat engaged after 0.1 s (pandad.cc:424) but the panda withdraws only after the engaged-mismatch count, about 3 s (panda main.c:226-232, SWF-014.C2); 0.3 s since panda f4803c5, reference build, after BL-006 (TSR-307(a))</t>
           </r>
           <r>
             <rPr>
@@ -18636,7 +18636,7 @@
               <color rgb="001B2430"/>
               <sz val="10"/>
             </rPr>
-            <t>PCM cruise stays engaged; the panda keeps controls allowed until the heartbeat-mismatch revoke (about 3 s)</t>
+            <t>PCM cruise stays engaged; the panda keeps controls allowed until the heartbeat-mismatch revoke (about 3 s at BL-006; since panda f4803c5, reference build, after BL-006, 0.3 s after the first not-engaged heartbeat, with the panda siren 0.5 s after it while cruise stays on, TSR-307(a), TSR-516(c))</t>
           </r>
           <r>
             <rPr>
@@ -32268,7 +32268,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;LSW FMEA — safety-relevant software elements · rev 1.7 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;LSW FMEA — safety-relevant software elements · rev 1.8 · BL-006&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>